<commit_message>
tablas para articulo formato de lineas y tecto ajustado
</commit_message>
<xml_diff>
--- a/excel_tables/tablas_valores_representativos_para_docx_acentos_corregidos.xlsx
+++ b/excel_tables/tablas_valores_representativos_para_docx_acentos_corregidos.xlsx
@@ -36,20 +36,15 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9EAF7"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -57,16 +52,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -460,6 +463,17 @@
           <t>Tabla 1. Valores representativos por tipo de muestra sólida</t>
         </is>
       </c>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
+      <c r="K1" s="1" t="n"/>
+      <c r="L1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -616,32 +630,32 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n"/>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
-      <c r="F5" s="3" t="n"/>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="3" t="n"/>
-      <c r="I5" s="3" t="n"/>
-      <c r="J5" s="3" t="n"/>
-      <c r="K5" s="3" t="n"/>
-      <c r="L5" s="3" t="n"/>
+      <c r="A5" s="4" t="n"/>
+      <c r="B5" s="4" t="n"/>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="n"/>
+      <c r="I5" s="4" t="n"/>
+      <c r="J5" s="4" t="n"/>
+      <c r="K5" s="4" t="n"/>
+      <c r="L5" s="4" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n"/>
-      <c r="B6" s="3" t="n"/>
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
-      <c r="F6" s="3" t="n"/>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
-      <c r="I6" s="3" t="n"/>
-      <c r="J6" s="3" t="n"/>
-      <c r="K6" s="3" t="n"/>
-      <c r="L6" s="3" t="n"/>
+      <c r="A6" s="4" t="n"/>
+      <c r="B6" s="4" t="n"/>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="n"/>
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="4" t="n"/>
+      <c r="I6" s="4" t="n"/>
+      <c r="J6" s="4" t="n"/>
+      <c r="K6" s="4" t="n"/>
+      <c r="L6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -856,32 +870,32 @@
       <c r="L12" s="3" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="n"/>
-      <c r="B13" s="3" t="n"/>
-      <c r="C13" s="3" t="n"/>
-      <c r="D13" s="3" t="n"/>
-      <c r="E13" s="3" t="n"/>
-      <c r="F13" s="3" t="n"/>
-      <c r="G13" s="3" t="n"/>
-      <c r="H13" s="3" t="n"/>
-      <c r="I13" s="3" t="n"/>
-      <c r="J13" s="3" t="n"/>
-      <c r="K13" s="3" t="n"/>
-      <c r="L13" s="3" t="n"/>
+      <c r="A13" s="4" t="n"/>
+      <c r="B13" s="4" t="n"/>
+      <c r="C13" s="4" t="n"/>
+      <c r="D13" s="4" t="n"/>
+      <c r="E13" s="4" t="n"/>
+      <c r="F13" s="4" t="n"/>
+      <c r="G13" s="4" t="n"/>
+      <c r="H13" s="4" t="n"/>
+      <c r="I13" s="4" t="n"/>
+      <c r="J13" s="4" t="n"/>
+      <c r="K13" s="4" t="n"/>
+      <c r="L13" s="4" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="n"/>
-      <c r="B14" s="3" t="n"/>
-      <c r="C14" s="3" t="n"/>
-      <c r="D14" s="3" t="n"/>
-      <c r="E14" s="3" t="n"/>
-      <c r="F14" s="3" t="n"/>
-      <c r="G14" s="3" t="n"/>
-      <c r="H14" s="3" t="n"/>
-      <c r="I14" s="3" t="n"/>
-      <c r="J14" s="3" t="n"/>
-      <c r="K14" s="3" t="n"/>
-      <c r="L14" s="3" t="n"/>
+      <c r="A14" s="4" t="n"/>
+      <c r="B14" s="4" t="n"/>
+      <c r="C14" s="4" t="n"/>
+      <c r="D14" s="4" t="n"/>
+      <c r="E14" s="4" t="n"/>
+      <c r="F14" s="4" t="n"/>
+      <c r="G14" s="4" t="n"/>
+      <c r="H14" s="4" t="n"/>
+      <c r="I14" s="4" t="n"/>
+      <c r="J14" s="4" t="n"/>
+      <c r="K14" s="4" t="n"/>
+      <c r="L14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
@@ -1127,6 +1141,15 @@
           <t>Contenido de masa seca y sólidos volátiles por muestra</t>
         </is>
       </c>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1363,6 +1386,14 @@
           <t>Nitrógeno total por muestra individual</t>
         </is>
       </c>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1390,6 +1421,10 @@
           <t>Nitrógeno total (mg/kg)</t>
         </is>
       </c>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -1413,6 +1448,10 @@
       <c r="E3" s="3" t="n">
         <v>24100</v>
       </c>
+      <c r="F3" s="3" t="n"/>
+      <c r="G3" s="3" t="n"/>
+      <c r="H3" s="3" t="n"/>
+      <c r="I3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -1436,6 +1475,10 @@
       <c r="E4" s="3" t="n">
         <v>24400</v>
       </c>
+      <c r="F4" s="3" t="n"/>
+      <c r="G4" s="3" t="n"/>
+      <c r="H4" s="3" t="n"/>
+      <c r="I4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -1459,6 +1502,10 @@
       <c r="E5" s="3" t="n">
         <v>71.90600000000001</v>
       </c>
+      <c r="F5" s="3" t="n"/>
+      <c r="G5" s="3" t="n"/>
+      <c r="H5" s="3" t="n"/>
+      <c r="I5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -1482,6 +1529,10 @@
       <c r="E6" s="3" t="n">
         <v>71.809</v>
       </c>
+      <c r="F6" s="3" t="n"/>
+      <c r="G6" s="3" t="n"/>
+      <c r="H6" s="3" t="n"/>
+      <c r="I6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -1505,6 +1556,10 @@
       <c r="E7" s="3" t="n">
         <v>109.76</v>
       </c>
+      <c r="F7" s="3" t="n"/>
+      <c r="G7" s="3" t="n"/>
+      <c r="H7" s="3" t="n"/>
+      <c r="I7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -1528,6 +1583,10 @@
       <c r="E8" s="3" t="n">
         <v>118.92</v>
       </c>
+      <c r="F8" s="3" t="n"/>
+      <c r="G8" s="3" t="n"/>
+      <c r="H8" s="3" t="n"/>
+      <c r="I8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -1551,6 +1610,10 @@
       <c r="E9" s="3" t="n">
         <v>4033.333</v>
       </c>
+      <c r="F9" s="3" t="n"/>
+      <c r="G9" s="3" t="n"/>
+      <c r="H9" s="3" t="n"/>
+      <c r="I9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1574,20 +1637,32 @@
       <c r="E10" s="3" t="n">
         <v>3400</v>
       </c>
+      <c r="F10" s="3" t="n"/>
+      <c r="G10" s="3" t="n"/>
+      <c r="H10" s="3" t="n"/>
+      <c r="I10" s="3" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n"/>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="3" t="n"/>
+      <c r="A11" s="4" t="n"/>
+      <c r="B11" s="4" t="n"/>
+      <c r="C11" s="4" t="n"/>
+      <c r="D11" s="4" t="n"/>
+      <c r="E11" s="4" t="n"/>
+      <c r="F11" s="4" t="n"/>
+      <c r="G11" s="4" t="n"/>
+      <c r="H11" s="4" t="n"/>
+      <c r="I11" s="4" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="n"/>
-      <c r="B12" s="3" t="n"/>
-      <c r="C12" s="3" t="n"/>
-      <c r="D12" s="3" t="n"/>
-      <c r="E12" s="3" t="n"/>
+      <c r="A12" s="4" t="n"/>
+      <c r="B12" s="4" t="n"/>
+      <c r="C12" s="4" t="n"/>
+      <c r="D12" s="4" t="n"/>
+      <c r="E12" s="4" t="n"/>
+      <c r="F12" s="4" t="n"/>
+      <c r="G12" s="4" t="n"/>
+      <c r="H12" s="4" t="n"/>
+      <c r="I12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
@@ -1599,6 +1674,10 @@
       <c r="C13" s="1" t="n"/>
       <c r="D13" s="1" t="n"/>
       <c r="E13" s="1" t="n"/>
+      <c r="F13" s="1" t="n"/>
+      <c r="G13" s="1" t="n"/>
+      <c r="H13" s="1" t="n"/>
+      <c r="I13" s="1" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">

</xml_diff>

<commit_message>
tablas para articulo con nombres tipo 1 y 2
</commit_message>
<xml_diff>
--- a/excel_tables/tablas_valores_representativos_para_docx_acentos_corregidos.xlsx
+++ b/excel_tables/tablas_valores_representativos_para_docx_acentos_corregidos.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,11 +29,15 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
-      <sz val="12"/>
+      <sz val="8"/>
     </font>
     <font>
       <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="8"/>
     </font>
   </fonts>
   <fills count="2">
@@ -63,13 +67,13 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -438,23 +442,23 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
-    <col width="34" customWidth="1" min="10" max="10"/>
-    <col width="34" customWidth="1" min="11" max="11"/>
-    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="6.5" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="7.5" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="7.5" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="6.5" customWidth="1" min="10" max="10"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
+    <col width="6" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -728,7 +732,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>A1 - Estiércol fresco</t>
+          <t>Estiércol fresco 1</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -764,7 +768,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>A2 - Estiércol fresco</t>
+          <t>Estiércol fresco 2</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -800,7 +804,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>B1 - Estiércol precompostado</t>
+          <t>Estiércol precompostado 1</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -836,7 +840,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>B2 - Estiércol precompostado</t>
+          <t>Estiércol precompostado 2</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1110,7 +1114,8 @@
       <c r="L20" s="3" t="n"/>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="1" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1118,21 +1123,21 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
-    <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1206,7 +1211,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>Estiércol fresco 1</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -1244,7 +1249,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>Estiércol fresco 2</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -1282,7 +1287,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>B1</t>
+          <t>Estiércol precompostado 1</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -1320,7 +1325,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>Estiércol precompostado 2</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -1356,7 +1361,8 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="1" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1364,20 +1370,20 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="27" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1859,7 +1865,8 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="1" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1867,12 +1874,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="120" customWidth="1" min="1" max="1"/>
+    <col width="85" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1892,7 +1899,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>El contenido de masa seca representativo por muestra corresponde al promedio de las réplicas agrupadas por código base de muestra (por ejemplo, A1, A2, B1, B2).</t>
+          <t>El contenido de masa seca representativo por muestra corresponde al promedio de las réplicas agrupadas por muestra de estiércol fresco o estiércol precompostado.</t>
         </is>
       </c>
     </row>
@@ -1918,6 +1925,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="1" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
prosa y tabla de articulo
</commit_message>
<xml_diff>
--- a/excel_tables/tablas_valores_representativos_para_docx_acentos_corregidos.xlsx
+++ b/excel_tables/tablas_valores_representativos_para_docx_acentos_corregidos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mateo\Downloads\LCA_IPCC_MANURE_TURRIALBA_UCR\excel_tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F50AAF9-E0B7-4C9F-84D4-A4F87B1838F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_F34DDC84090D52E1E418867E5A9D0AF8B869AE3F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,25 +18,12 @@
     <sheet name="Nitrógeno total" sheetId="3" r:id="rId3"/>
     <sheet name="Notas" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="121">
   <si>
     <t>Tabla 1. Valores representativos por tipo de muestra sólida</t>
   </si>
@@ -65,6 +52,9 @@
     <t>Desviación estándar de sólidos volátiles (%)</t>
   </si>
   <si>
+    <t>Precisión instrumental de masa</t>
+  </si>
+  <si>
     <t>Fecha de análisis de nitrógeno</t>
   </si>
   <si>
@@ -77,6 +67,9 @@
     <t>Nitrógeno total promedio (mg/kg)</t>
   </si>
   <si>
+    <t>Precisión reportada de nitrógeno</t>
+  </si>
+  <si>
     <t>A - estiércol fresco</t>
   </si>
   <si>
@@ -86,18 +79,60 @@
     <t>10/11/2025</t>
   </si>
   <si>
+    <t>14.230</t>
+  </si>
+  <si>
+    <t>0.621</t>
+  </si>
+  <si>
+    <t>85.877</t>
+  </si>
+  <si>
+    <t>0.668</t>
+  </si>
+  <si>
+    <t>±0.1 mg</t>
+  </si>
+  <si>
     <t>19/11/2025</t>
   </si>
   <si>
+    <t>0.37</t>
+  </si>
+  <si>
+    <t>3716.67</t>
+  </si>
+  <si>
+    <t>±0.01</t>
+  </si>
+  <si>
     <t>B - estiércol precompostado</t>
   </si>
   <si>
     <t>Estiércol precompostado</t>
   </si>
   <si>
+    <t>22.407</t>
+  </si>
+  <si>
+    <t>3.927</t>
+  </si>
+  <si>
+    <t>70.959</t>
+  </si>
+  <si>
+    <t>4.256</t>
+  </si>
+  <si>
     <t>21/11/2025</t>
   </si>
   <si>
+    <t>2.42</t>
+  </si>
+  <si>
+    <t>24250.00</t>
+  </si>
+  <si>
     <t>Tabla 2. Contenido de masa seca y sólidos volátiles por muestra</t>
   </si>
   <si>
@@ -116,15 +151,87 @@
     <t>Estiércol fresco 1</t>
   </si>
   <si>
+    <t>13.791</t>
+  </si>
+  <si>
+    <t>0.110</t>
+  </si>
+  <si>
+    <t>0.795</t>
+  </si>
+  <si>
+    <t>85.405</t>
+  </si>
+  <si>
+    <t>0.783</t>
+  </si>
+  <si>
+    <t>0.917</t>
+  </si>
+  <si>
     <t>Estiércol fresco 2</t>
   </si>
   <si>
+    <t>14.669</t>
+  </si>
+  <si>
+    <t>0.339</t>
+  </si>
+  <si>
+    <t>2.313</t>
+  </si>
+  <si>
+    <t>86.349</t>
+  </si>
+  <si>
+    <t>1.679</t>
+  </si>
+  <si>
+    <t>1.945</t>
+  </si>
+  <si>
     <t>Estiércol precompostado 1</t>
   </si>
   <si>
+    <t>19.630</t>
+  </si>
+  <si>
+    <t>0.239</t>
+  </si>
+  <si>
+    <t>1.216</t>
+  </si>
+  <si>
+    <t>73.968</t>
+  </si>
+  <si>
+    <t>1.847</t>
+  </si>
+  <si>
+    <t>2.497</t>
+  </si>
+  <si>
     <t>Estiércol precompostado 2</t>
   </si>
   <si>
+    <t>25.184</t>
+  </si>
+  <si>
+    <t>0.298</t>
+  </si>
+  <si>
+    <t>1.182</t>
+  </si>
+  <si>
+    <t>67.949</t>
+  </si>
+  <si>
+    <t>0.304</t>
+  </si>
+  <si>
+    <t>0.448</t>
+  </si>
+  <si>
     <t>Tabla 3. Nitrógeno total representativo por muestra o tratamiento</t>
   </si>
   <si>
@@ -146,18 +253,51 @@
     <t>Valor máximo de nitrógeno total (mg/kg)</t>
   </si>
   <si>
+    <t>3400.00</t>
+  </si>
+  <si>
+    <t>4033.33</t>
+  </si>
+  <si>
     <t>Líquido: agua verde</t>
   </si>
   <si>
+    <t>0.01</t>
+  </si>
+  <si>
+    <t>71.86</t>
+  </si>
+  <si>
+    <t>71.81</t>
+  </si>
+  <si>
+    <t>71.91</t>
+  </si>
+  <si>
     <t>Líquido: purines</t>
   </si>
   <si>
     <t>28/11/2025</t>
   </si>
   <si>
+    <t>114.34</t>
+  </si>
+  <si>
+    <t>109.76</t>
+  </si>
+  <si>
+    <t>118.92</t>
+  </si>
+  <si>
     <t>Sólido precompostado</t>
   </si>
   <si>
+    <t>24100.00</t>
+  </si>
+  <si>
+    <t>24400.00</t>
+  </si>
+  <si>
     <t>Contenido de masa seca y sólidos volátiles por muestra</t>
   </si>
   <si>
@@ -179,9 +319,15 @@
     <t>CN</t>
   </si>
   <si>
+    <t>2.41</t>
+  </si>
+  <si>
     <t>SOL: PRECOMPOSTADO 2</t>
   </si>
   <si>
+    <t>2.44</t>
+  </si>
+  <si>
     <t>LIQ: AGUA VERDE 1</t>
   </si>
   <si>
@@ -206,9 +352,15 @@
     <t>N total (Kjeldahl)</t>
   </si>
   <si>
+    <t>0.40</t>
+  </si>
+  <si>
     <t>ESTIERCOL FRESCO 3</t>
   </si>
   <si>
+    <t>0.34</t>
+  </si>
+  <si>
     <t>Nitrógeno total representativo por muestra o tratamiento</t>
   </si>
   <si>
@@ -222,6 +374,12 @@
   </si>
   <si>
     <t>Los sólidos volátiles se calcularon como 100 menos el porcentaje de cenizas, en base seca.</t>
+  </si>
+  <si>
+    <t>Para masa seca y sólidos volátiles, la precisión instrumental corresponde a la balanza analítica utilizada: ±0.1 mg.</t>
+  </si>
+  <si>
+    <t>Para nitrógeno total, los resultados de laboratorio se reportan con dos decimales; por eso se indica una precisión reportada de ±0.01 en la unidad de la columna.</t>
   </si>
   <si>
     <t>El nitrógeno total representativo proviene de processed/CIA_samples_table_v6_treatment_summary.csv y corresponde al promedio por tratamiento usado por el script.</t>
@@ -605,23 +763,24 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.453125" customWidth="1"/>
-    <col min="2" max="2" width="9" customWidth="1"/>
-    <col min="3" max="3" width="7" customWidth="1"/>
-    <col min="4" max="4" width="6.453125" customWidth="1"/>
-    <col min="5" max="5" width="8" customWidth="1"/>
-    <col min="6" max="6" width="7.453125" customWidth="1"/>
-    <col min="7" max="7" width="8" customWidth="1"/>
-    <col min="8" max="8" width="7.453125" customWidth="1"/>
-    <col min="9" max="9" width="7" customWidth="1"/>
-    <col min="10" max="10" width="6.453125" customWidth="1"/>
-    <col min="11" max="12" width="6" customWidth="1"/>
+    <col min="1" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="6" customWidth="1"/>
+    <col min="4" max="4" width="5.453125" customWidth="1"/>
+    <col min="5" max="5" width="6.453125" customWidth="1"/>
+    <col min="6" max="6" width="6" customWidth="1"/>
+    <col min="7" max="7" width="6.453125" customWidth="1"/>
+    <col min="8" max="8" width="6" customWidth="1"/>
+    <col min="9" max="9" width="5.453125" customWidth="1"/>
+    <col min="10" max="10" width="6" customWidth="1"/>
+    <col min="11" max="12" width="5.453125" customWidth="1"/>
+    <col min="13" max="13" width="6" customWidth="1"/>
+    <col min="14" max="14" width="5.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="84" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" ht="84" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -636,8 +795,10 @@
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
-    </row>
-    <row r="2" spans="1:12" ht="63" x14ac:dyDescent="0.35">
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+    </row>
+    <row r="2" spans="1:14" ht="84" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -674,84 +835,102 @@
       <c r="L2" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" ht="21" x14ac:dyDescent="0.35">
+      <c r="M2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="21" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D3" s="3">
         <v>2</v>
       </c>
-      <c r="E3" s="3">
-        <v>14.23</v>
-      </c>
-      <c r="F3" s="3">
-        <v>0.621</v>
-      </c>
-      <c r="G3" s="3">
-        <v>85.876999999999995</v>
-      </c>
-      <c r="H3" s="3">
-        <v>0.66800000000000004</v>
+      <c r="E3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>21</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J3" s="3">
+        <v>22</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="K3" s="3">
         <v>2</v>
       </c>
-      <c r="K3" s="3">
-        <v>0.372</v>
-      </c>
-      <c r="L3" s="3">
-        <v>3716.6669999999999</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" ht="31.5" x14ac:dyDescent="0.35">
+      <c r="L3" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ht="31.5" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>17</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>15</v>
       </c>
       <c r="D4" s="3">
         <v>2</v>
       </c>
-      <c r="E4" s="3">
-        <v>22.407</v>
-      </c>
-      <c r="F4" s="3">
-        <v>3.927</v>
-      </c>
-      <c r="G4" s="3">
-        <v>70.959000000000003</v>
-      </c>
-      <c r="H4" s="3">
-        <v>4.2560000000000002</v>
+      <c r="E4" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>32</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="J4" s="3">
+        <v>22</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="K4" s="3">
         <v>2</v>
       </c>
-      <c r="K4" s="3">
-        <v>2.4249999999999998</v>
-      </c>
-      <c r="L4" s="3">
-        <v>24250</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="L4" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="N4" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5" s="4"/>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
@@ -764,8 +943,10 @@
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
       <c r="L5" s="4"/>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M5" s="4"/>
+      <c r="N5" s="4"/>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" s="4"/>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -778,10 +959,12 @@
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
       <c r="L6" s="4"/>
-    </row>
-    <row r="7" spans="1:12" ht="96" x14ac:dyDescent="0.35">
+      <c r="M6" s="4"/>
+      <c r="N6" s="4"/>
+    </row>
+    <row r="7" spans="1:14" ht="96" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -794,16 +977,18 @@
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
-    </row>
-    <row r="8" spans="1:12" ht="84" x14ac:dyDescent="0.35">
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+    </row>
+    <row r="8" spans="1:14" ht="94.5" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>5</v>
@@ -812,7 +997,7 @@
         <v>6</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>7</v>
@@ -821,141 +1006,161 @@
         <v>8</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="J8" s="2"/>
+        <v>40</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
-    </row>
-    <row r="9" spans="1:12" ht="21" x14ac:dyDescent="0.35">
+      <c r="M8" s="2"/>
+      <c r="N8" s="2"/>
+    </row>
+    <row r="9" spans="1:14" ht="21" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C9" s="3">
         <v>3</v>
       </c>
-      <c r="D9" s="3">
-        <v>13.791</v>
-      </c>
-      <c r="E9" s="3">
-        <v>0.11</v>
-      </c>
-      <c r="F9" s="3">
-        <v>0.79500000000000004</v>
-      </c>
-      <c r="G9" s="3">
-        <v>85.405000000000001</v>
-      </c>
-      <c r="H9" s="3">
-        <v>0.78300000000000003</v>
-      </c>
-      <c r="I9" s="3">
-        <v>0.91700000000000004</v>
-      </c>
-      <c r="J9" s="3"/>
+      <c r="D9" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="K9" s="3"/>
       <c r="L9" s="3"/>
-    </row>
-    <row r="10" spans="1:12" ht="21" x14ac:dyDescent="0.35">
+      <c r="M9" s="3"/>
+      <c r="N9" s="3"/>
+    </row>
+    <row r="10" spans="1:14" ht="21" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>26</v>
+        <v>48</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C10" s="3">
         <v>3</v>
       </c>
-      <c r="D10" s="3">
-        <v>14.669</v>
-      </c>
-      <c r="E10" s="3">
-        <v>0.33900000000000002</v>
-      </c>
-      <c r="F10" s="3">
-        <v>2.3130000000000002</v>
-      </c>
-      <c r="G10" s="3">
-        <v>86.349000000000004</v>
-      </c>
-      <c r="H10" s="3">
-        <v>1.679</v>
-      </c>
-      <c r="I10" s="3">
-        <v>1.9450000000000001</v>
-      </c>
-      <c r="J10" s="3"/>
+      <c r="D10" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="K10" s="3"/>
       <c r="L10" s="3"/>
-    </row>
-    <row r="11" spans="1:12" ht="31.5" x14ac:dyDescent="0.35">
+      <c r="M10" s="3"/>
+      <c r="N10" s="3"/>
+    </row>
+    <row r="11" spans="1:14" ht="31.5" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C11" s="3">
         <v>3</v>
       </c>
-      <c r="D11" s="3">
-        <v>19.63</v>
-      </c>
-      <c r="E11" s="3">
-        <v>0.23899999999999999</v>
-      </c>
-      <c r="F11" s="3">
-        <v>1.216</v>
-      </c>
-      <c r="G11" s="3">
-        <v>73.968000000000004</v>
-      </c>
-      <c r="H11" s="3">
-        <v>1.847</v>
-      </c>
-      <c r="I11" s="3">
-        <v>2.4969999999999999</v>
-      </c>
-      <c r="J11" s="3"/>
+      <c r="D11" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="K11" s="3"/>
       <c r="L11" s="3"/>
-    </row>
-    <row r="12" spans="1:12" ht="31.5" x14ac:dyDescent="0.35">
+      <c r="M11" s="3"/>
+      <c r="N11" s="3"/>
+    </row>
+    <row r="12" spans="1:14" ht="31.5" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>28</v>
+        <v>62</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C12" s="3">
         <v>3</v>
       </c>
-      <c r="D12" s="3">
-        <v>25.184000000000001</v>
-      </c>
-      <c r="E12" s="3">
-        <v>0.29799999999999999</v>
-      </c>
-      <c r="F12" s="3">
-        <v>1.1819999999999999</v>
-      </c>
-      <c r="G12" s="3">
-        <v>67.948999999999998</v>
-      </c>
-      <c r="H12" s="3">
-        <v>0.30399999999999999</v>
-      </c>
-      <c r="I12" s="3">
-        <v>0.44800000000000001</v>
-      </c>
-      <c r="J12" s="3"/>
+      <c r="D12" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="K12" s="3"/>
       <c r="L12" s="3"/>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M12" s="3"/>
+      <c r="N12" s="3"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A13" s="4"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -968,8 +1173,10 @@
       <c r="J13" s="4"/>
       <c r="K13" s="4"/>
       <c r="L13" s="4"/>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M13" s="4"/>
+      <c r="N13" s="4"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" s="4"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -982,10 +1189,12 @@
       <c r="J14" s="4"/>
       <c r="K14" s="4"/>
       <c r="L14" s="4"/>
-    </row>
-    <row r="15" spans="1:12" ht="96" x14ac:dyDescent="0.35">
+      <c r="M14" s="4"/>
+      <c r="N14" s="4"/>
+    </row>
+    <row r="15" spans="1:14" ht="96" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
-        <v>29</v>
+        <v>69</v>
       </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -998,166 +1207,188 @@
       <c r="J15" s="1"/>
       <c r="K15" s="1"/>
       <c r="L15" s="1"/>
-    </row>
-    <row r="16" spans="1:12" ht="63" x14ac:dyDescent="0.35">
+      <c r="M15" s="1"/>
+      <c r="N15" s="1"/>
+    </row>
+    <row r="16" spans="1:14" ht="84" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>31</v>
+        <v>71</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>32</v>
+        <v>72</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>33</v>
+        <v>73</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="J16" s="2"/>
+        <v>75</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="K16" s="2"/>
       <c r="L16" s="2"/>
-    </row>
-    <row r="17" spans="1:12" ht="21" x14ac:dyDescent="0.35">
+      <c r="M16" s="2"/>
+      <c r="N16" s="2"/>
+    </row>
+    <row r="17" spans="1:14" ht="21" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="C17" s="3">
         <v>2</v>
       </c>
-      <c r="D17" s="3">
-        <v>0.372</v>
-      </c>
-      <c r="E17" s="3">
-        <v>3716.6669999999999</v>
-      </c>
-      <c r="F17" s="3">
-        <v>0.372</v>
-      </c>
-      <c r="G17" s="3">
-        <v>3716.6669999999999</v>
-      </c>
-      <c r="H17" s="3">
-        <v>3400</v>
-      </c>
-      <c r="I17" s="3">
-        <v>4033.3330000000001</v>
-      </c>
-      <c r="J17" s="3"/>
+      <c r="D17" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>26</v>
+      </c>
       <c r="K17" s="3"/>
       <c r="L17" s="3"/>
-    </row>
-    <row r="18" spans="1:12" ht="21" x14ac:dyDescent="0.35">
+      <c r="M17" s="3"/>
+      <c r="N17" s="3"/>
+    </row>
+    <row r="18" spans="1:14" ht="21" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
-        <v>36</v>
+        <v>78</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="C18" s="3">
         <v>2</v>
       </c>
-      <c r="D18" s="3">
-        <v>7.0000000000000001E-3</v>
-      </c>
-      <c r="E18" s="3">
-        <v>71.858000000000004</v>
-      </c>
-      <c r="F18" s="3">
-        <v>7.0000000000000001E-3</v>
-      </c>
-      <c r="G18" s="3">
-        <v>71.858000000000004</v>
-      </c>
-      <c r="H18" s="3">
-        <v>71.808999999999997</v>
-      </c>
-      <c r="I18" s="3">
-        <v>71.906000000000006</v>
-      </c>
-      <c r="J18" s="3"/>
+      <c r="D18" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="J18" s="3" t="s">
+        <v>26</v>
+      </c>
       <c r="K18" s="3"/>
       <c r="L18" s="3"/>
-    </row>
-    <row r="19" spans="1:12" ht="21" x14ac:dyDescent="0.35">
+      <c r="M18" s="3"/>
+      <c r="N18" s="3"/>
+    </row>
+    <row r="19" spans="1:14" ht="21" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>37</v>
+        <v>83</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>38</v>
+        <v>84</v>
       </c>
       <c r="C19" s="3">
         <v>2</v>
       </c>
-      <c r="D19" s="3">
-        <v>1.0999999999999999E-2</v>
-      </c>
-      <c r="E19" s="3">
-        <v>114.34</v>
-      </c>
-      <c r="F19" s="3">
-        <v>1.0999999999999999E-2</v>
-      </c>
-      <c r="G19" s="3">
-        <v>114.34</v>
-      </c>
-      <c r="H19" s="3">
-        <v>109.76</v>
-      </c>
-      <c r="I19" s="3">
-        <v>118.92</v>
-      </c>
-      <c r="J19" s="3"/>
+      <c r="D19" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="J19" s="3" t="s">
+        <v>26</v>
+      </c>
       <c r="K19" s="3"/>
       <c r="L19" s="3"/>
-    </row>
-    <row r="20" spans="1:12" ht="31.5" x14ac:dyDescent="0.35">
+      <c r="M19" s="3"/>
+      <c r="N19" s="3"/>
+    </row>
+    <row r="20" spans="1:14" ht="31.5" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
-        <v>39</v>
+        <v>88</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="C20" s="3">
         <v>2</v>
       </c>
-      <c r="D20" s="3">
-        <v>2.4249999999999998</v>
-      </c>
-      <c r="E20" s="3">
-        <v>24250</v>
-      </c>
-      <c r="F20" s="3">
-        <v>2.4249999999999998</v>
-      </c>
-      <c r="G20" s="3">
-        <v>24250</v>
-      </c>
-      <c r="H20" s="3">
-        <v>24100</v>
-      </c>
-      <c r="I20" s="3">
-        <v>24400</v>
-      </c>
-      <c r="J20" s="3"/>
+      <c r="D20" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="J20" s="3" t="s">
+        <v>26</v>
+      </c>
       <c r="K20" s="3"/>
       <c r="L20" s="3"/>
+      <c r="M20" s="3"/>
+      <c r="N20" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
@@ -1170,22 +1401,22 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="7" customWidth="1"/>
-    <col min="2" max="2" width="9" customWidth="1"/>
-    <col min="3" max="3" width="7" customWidth="1"/>
-    <col min="4" max="4" width="6" customWidth="1"/>
-    <col min="5" max="5" width="8" customWidth="1"/>
-    <col min="6" max="7" width="7" customWidth="1"/>
-    <col min="8" max="8" width="8" customWidth="1"/>
-    <col min="9" max="10" width="7" customWidth="1"/>
+    <col min="1" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="6.453125" customWidth="1"/>
+    <col min="4" max="4" width="5.453125" customWidth="1"/>
+    <col min="5" max="5" width="6.453125" customWidth="1"/>
+    <col min="6" max="7" width="6" customWidth="1"/>
+    <col min="8" max="8" width="6.453125" customWidth="1"/>
+    <col min="9" max="10" width="6" customWidth="1"/>
+    <col min="11" max="11" width="5.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="96" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" ht="84" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>40</v>
+        <v>91</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1196,8 +1427,9 @@
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
-    </row>
-    <row r="2" spans="1:10" ht="63" x14ac:dyDescent="0.35">
+      <c r="K1" s="1"/>
+    </row>
+    <row r="2" spans="1:11" ht="84" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -1205,10 +1437,10 @@
         <v>2</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>5</v>
@@ -1217,7 +1449,7 @@
         <v>6</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>7</v>
@@ -1226,135 +1458,150 @@
         <v>8</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="21" x14ac:dyDescent="0.35">
+        <v>40</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="21" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D3" s="3">
         <v>3</v>
       </c>
-      <c r="E3" s="3">
-        <v>13.791</v>
-      </c>
-      <c r="F3" s="3">
-        <v>0.11</v>
-      </c>
-      <c r="G3" s="3">
-        <v>0.79500000000000004</v>
-      </c>
-      <c r="H3" s="3">
-        <v>85.405000000000001</v>
-      </c>
-      <c r="I3" s="3">
-        <v>0.78300000000000003</v>
-      </c>
-      <c r="J3" s="3">
-        <v>0.91700000000000004</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="E3" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="21" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>26</v>
+        <v>48</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D4" s="3">
         <v>3</v>
       </c>
-      <c r="E4" s="3">
-        <v>14.669</v>
-      </c>
-      <c r="F4" s="3">
-        <v>0.33900000000000002</v>
-      </c>
-      <c r="G4" s="3">
-        <v>2.3130000000000002</v>
-      </c>
-      <c r="H4" s="3">
-        <v>86.349000000000004</v>
-      </c>
-      <c r="I4" s="3">
-        <v>1.679</v>
-      </c>
-      <c r="J4" s="3">
-        <v>1.9450000000000001</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="31.5" x14ac:dyDescent="0.35">
+      <c r="E4" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="31.5" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D5" s="3">
         <v>3</v>
       </c>
-      <c r="E5" s="3">
-        <v>19.63</v>
-      </c>
-      <c r="F5" s="3">
-        <v>0.23899999999999999</v>
-      </c>
-      <c r="G5" s="3">
-        <v>1.216</v>
-      </c>
-      <c r="H5" s="3">
-        <v>73.968000000000004</v>
-      </c>
-      <c r="I5" s="3">
-        <v>1.847</v>
-      </c>
-      <c r="J5" s="3">
-        <v>2.4969999999999999</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="31.5" x14ac:dyDescent="0.35">
+      <c r="E5" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="31.5" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>18</v>
-      </c>
       <c r="C6" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D6" s="3">
         <v>3</v>
       </c>
-      <c r="E6" s="3">
-        <v>25.184000000000001</v>
-      </c>
-      <c r="F6" s="3">
-        <v>0.29799999999999999</v>
-      </c>
-      <c r="G6" s="3">
-        <v>1.1819999999999999</v>
-      </c>
-      <c r="H6" s="3">
-        <v>67.948999999999998</v>
-      </c>
-      <c r="I6" s="3">
-        <v>0.30399999999999999</v>
-      </c>
-      <c r="J6" s="3">
-        <v>0.44800000000000001</v>
+      <c r="E6" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -1368,21 +1615,22 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11" customWidth="1"/>
-    <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="3" max="4" width="7" customWidth="1"/>
-    <col min="5" max="5" width="8" customWidth="1"/>
-    <col min="6" max="6" width="7" customWidth="1"/>
-    <col min="7" max="7" width="8" customWidth="1"/>
-    <col min="8" max="9" width="7" customWidth="1"/>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="2" width="9" customWidth="1"/>
+    <col min="3" max="4" width="6.453125" customWidth="1"/>
+    <col min="5" max="5" width="7" customWidth="1"/>
+    <col min="6" max="6" width="5.453125" customWidth="1"/>
+    <col min="7" max="7" width="6.453125" customWidth="1"/>
+    <col min="8" max="8" width="7" customWidth="1"/>
+    <col min="9" max="10" width="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="48" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="48" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>41</v>
+        <v>92</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1392,197 +1640,225 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
-    </row>
-    <row r="2" spans="1:9" ht="31.5" x14ac:dyDescent="0.35">
+      <c r="J1" s="1"/>
+    </row>
+    <row r="2" spans="1:10" ht="63" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>42</v>
+        <v>93</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>43</v>
+        <v>94</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="F2" s="2"/>
+        <v>95</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
-    </row>
-    <row r="3" spans="1:9" ht="31.5" x14ac:dyDescent="0.35">
+      <c r="J2" s="2"/>
+    </row>
+    <row r="3" spans="1:10" ht="31.5" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>45</v>
+        <v>96</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>46</v>
+        <v>97</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D3" s="3">
-        <v>2.41</v>
-      </c>
-      <c r="E3" s="3">
-        <v>24100</v>
-      </c>
-      <c r="F3" s="3"/>
+        <v>33</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>26</v>
+      </c>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
-    </row>
-    <row r="4" spans="1:9" ht="31.5" x14ac:dyDescent="0.35">
+      <c r="J3" s="3"/>
+    </row>
+    <row r="4" spans="1:10" ht="31.5" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>47</v>
+        <v>99</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>46</v>
+        <v>97</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D4" s="3">
-        <v>2.44</v>
-      </c>
-      <c r="E4" s="3">
-        <v>24400</v>
-      </c>
-      <c r="F4" s="3"/>
+        <v>33</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>26</v>
+      </c>
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
-    </row>
-    <row r="5" spans="1:9" ht="31.5" x14ac:dyDescent="0.35">
+      <c r="J4" s="3"/>
+    </row>
+    <row r="5" spans="1:10" ht="31.5" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>48</v>
+        <v>101</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>49</v>
+        <v>102</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" s="3">
-        <v>7.0000000000000001E-3</v>
-      </c>
-      <c r="E5" s="3">
-        <v>71.906000000000006</v>
-      </c>
-      <c r="F5" s="3"/>
+        <v>33</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>26</v>
+      </c>
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
-    </row>
-    <row r="6" spans="1:9" ht="31.5" x14ac:dyDescent="0.35">
+      <c r="J5" s="3"/>
+    </row>
+    <row r="6" spans="1:10" ht="31.5" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>50</v>
+        <v>103</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>49</v>
+        <v>102</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D6" s="3">
-        <v>7.0000000000000001E-3</v>
-      </c>
-      <c r="E6" s="3">
-        <v>71.808999999999997</v>
-      </c>
-      <c r="F6" s="3"/>
+        <v>33</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>26</v>
+      </c>
       <c r="G6" s="3"/>
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
-    </row>
-    <row r="7" spans="1:9" ht="21" x14ac:dyDescent="0.35">
+      <c r="J6" s="3"/>
+    </row>
+    <row r="7" spans="1:10" ht="31.5" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>51</v>
+        <v>104</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>52</v>
+        <v>105</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="D7" s="3">
-        <v>1.0999999999999999E-2</v>
-      </c>
-      <c r="E7" s="3">
-        <v>109.76</v>
-      </c>
-      <c r="F7" s="3"/>
+        <v>84</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>26</v>
+      </c>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
-    </row>
-    <row r="8" spans="1:9" ht="21" x14ac:dyDescent="0.35">
+      <c r="J7" s="3"/>
+    </row>
+    <row r="8" spans="1:10" ht="31.5" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>53</v>
+        <v>106</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>52</v>
+        <v>105</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="D8" s="3">
-        <v>1.2E-2</v>
-      </c>
-      <c r="E8" s="3">
-        <v>118.92</v>
-      </c>
-      <c r="F8" s="3"/>
+        <v>84</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>26</v>
+      </c>
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
-    </row>
-    <row r="9" spans="1:9" ht="21" x14ac:dyDescent="0.35">
+      <c r="J8" s="3"/>
+    </row>
+    <row r="9" spans="1:10" ht="21" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>55</v>
+        <v>108</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9" s="3">
-        <v>0.40300000000000002</v>
-      </c>
-      <c r="E9" s="3">
-        <v>4033.3330000000001</v>
-      </c>
-      <c r="F9" s="3"/>
+        <v>23</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>26</v>
+      </c>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
-    </row>
-    <row r="10" spans="1:9" ht="21" x14ac:dyDescent="0.35">
+      <c r="J9" s="3"/>
+    </row>
+    <row r="10" spans="1:10" ht="21" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>56</v>
+        <v>110</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>55</v>
+        <v>108</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D10" s="3">
-        <v>0.34</v>
-      </c>
-      <c r="E10" s="3">
-        <v>3400</v>
-      </c>
-      <c r="F10" s="3"/>
+        <v>23</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>26</v>
+      </c>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J10" s="3"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -1592,8 +1868,9 @@
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J11" s="4"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="4"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
@@ -1603,10 +1880,11 @@
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
-    </row>
-    <row r="13" spans="1:9" ht="60" x14ac:dyDescent="0.35">
+      <c r="J12" s="4"/>
+    </row>
+    <row r="13" spans="1:10" ht="72" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
-        <v>57</v>
+        <v>112</v>
       </c>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -1616,150 +1894,166 @@
       <c r="G13" s="1"/>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
-    </row>
-    <row r="14" spans="1:9" ht="63" x14ac:dyDescent="0.35">
+      <c r="J13" s="1"/>
+    </row>
+    <row r="14" spans="1:10" ht="73.5" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>31</v>
+        <v>71</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>32</v>
+        <v>72</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>33</v>
+        <v>73</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+        <v>75</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="C15" s="3">
         <v>2</v>
       </c>
-      <c r="D15" s="3">
-        <v>0.372</v>
-      </c>
-      <c r="E15" s="3">
-        <v>3716.6669999999999</v>
-      </c>
-      <c r="F15" s="3">
-        <v>0.372</v>
-      </c>
-      <c r="G15" s="3">
-        <v>3716.6669999999999</v>
-      </c>
-      <c r="H15" s="3">
-        <v>3400</v>
-      </c>
-      <c r="I15" s="3">
-        <v>4033.3330000000001</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="21" x14ac:dyDescent="0.35">
+      <c r="D15" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="21" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
-        <v>36</v>
+        <v>78</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="C16" s="3">
         <v>2</v>
       </c>
-      <c r="D16" s="3">
-        <v>7.0000000000000001E-3</v>
-      </c>
-      <c r="E16" s="3">
-        <v>71.858000000000004</v>
-      </c>
-      <c r="F16" s="3">
-        <v>7.0000000000000001E-3</v>
-      </c>
-      <c r="G16" s="3">
-        <v>71.858000000000004</v>
-      </c>
-      <c r="H16" s="3">
-        <v>71.808999999999997</v>
-      </c>
-      <c r="I16" s="3">
-        <v>71.906000000000006</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="D16" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="21" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>37</v>
+        <v>83</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>38</v>
+        <v>84</v>
       </c>
       <c r="C17" s="3">
         <v>2</v>
       </c>
-      <c r="D17" s="3">
-        <v>1.0999999999999999E-2</v>
-      </c>
-      <c r="E17" s="3">
-        <v>114.34</v>
-      </c>
-      <c r="F17" s="3">
-        <v>1.0999999999999999E-2</v>
-      </c>
-      <c r="G17" s="3">
-        <v>114.34</v>
-      </c>
-      <c r="H17" s="3">
-        <v>109.76</v>
-      </c>
-      <c r="I17" s="3">
-        <v>118.92</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" ht="21" x14ac:dyDescent="0.35">
+      <c r="D17" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="21" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
-        <v>39</v>
+        <v>88</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="C18" s="3">
         <v>2</v>
       </c>
-      <c r="D18" s="3">
-        <v>2.4249999999999998</v>
-      </c>
-      <c r="E18" s="3">
-        <v>24250</v>
-      </c>
-      <c r="F18" s="3">
-        <v>2.4249999999999998</v>
-      </c>
-      <c r="G18" s="3">
-        <v>24250</v>
-      </c>
-      <c r="H18" s="3">
-        <v>24100</v>
-      </c>
-      <c r="I18" s="3">
-        <v>24400</v>
+      <c r="D18" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="J18" s="3" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -1773,7 +2067,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="85" customWidth="1"/>
@@ -1781,32 +2075,42 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>58</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="21" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>59</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="21" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>60</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" ht="21" x14ac:dyDescent="0.35">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" ht="21" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>63</v>
+        <v>118</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="21" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>120</v>
       </c>
     </row>
   </sheetData>

</xml_diff>